<commit_message>
fix: keep long cell text in the status bar from crowding out the tabs
The selected cell's text could take up to 60% of the footer and squeeze
the sheet tabs, which matters most in a side-by-side comparison. Cap it
at 240 pixels with an ellipsis and the whole text on hover, let it give
way before the tabs do, and leave it out when the view is narrow.
</commit_message>
<xml_diff>
--- a/test/fixtures/many-sheets.xlsx
+++ b/test/fixtures/many-sheets.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t xml:space="preserve">Summary</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figures before March 2025 come from the old billing system and were converted at the average monthly exchange rate; later months use the rate on the invoice date. Forecast sheets assume the pricing approved in the Q4 2025 review.</t>
   </si>
 </sst>
 </file>
@@ -1553,6 +1556,11 @@
         <v>323</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: keep long cell text in the status bar from crowding out the tabs (#32)
The selected cell's text could take up to 60% of the footer and squeeze
the sheet tabs, which matters most in a side-by-side comparison. Cap it
at 240 pixels with an ellipsis and the whole text on hover, let it give
way before the tabs do, and leave it out when the view is narrow.
</commit_message>
<xml_diff>
--- a/test/fixtures/many-sheets.xlsx
+++ b/test/fixtures/many-sheets.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t xml:space="preserve">Summary</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figures before March 2025 come from the old billing system and were converted at the average monthly exchange rate; later months use the rate on the invoice date. Forecast sheets assume the pricing approved in the Q4 2025 review.</t>
   </si>
 </sst>
 </file>
@@ -1553,6 +1556,11 @@
         <v>323</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>